<commit_message>
Fix Excel compatibility with Numbers (macOS) and Google Sheets
- Removed emoji from Dashboard sheet name (caused parse error in Numbers)
- Removed DataLabelList from pie chart (generated invalid XML in some viewers)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/extracted.xlsx
+++ b/data/extracted.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="📊 Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="All Policies" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Expiry Alerts (&lt;=30d)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="By Status" sheetId="4" state="visible" r:id="rId4"/>
@@ -338,10 +338,6 @@
             </numRef>
           </val>
         </ser>
-        <dLbls>
-          <showCatName val="1"/>
-          <showPercent val="1"/>
-        </dLbls>
         <firstSliceAng val="0"/>
       </pieChart>
     </plotArea>

</xml_diff>

<commit_message>
feat: add FastAPI incremental upload and dashboard filters
</commit_message>
<xml_diff>
--- a/data/extracted.xlsx
+++ b/data/extracted.xlsx
@@ -20479,12 +20479,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>P6DED152PDA000109.pdf</t>
+          <t>P6DED152PDA000120.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>P6DED152PDA000109</t>
+          <t>P6DED152PDA000120</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -20494,7 +20494,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>D202160528</t>
+          <t>D202160551</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -20540,12 +20540,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>P6DED152PDA000112.pdf</t>
+          <t>P6DED152PDA000109.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>P6DED152PDA000112</t>
+          <t>P6DED152PDA000109</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -20555,7 +20555,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>D202160533</t>
+          <t>D202160528</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -20601,12 +20601,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>P6DED152PDA000120.pdf</t>
+          <t>P6DED152PDA000112.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>P6DED152PDA000120</t>
+          <t>P6DED152PDA000112</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -20616,7 +20616,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>D202160551</t>
+          <t>D202160533</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -20723,12 +20723,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014404.pdf</t>
+          <t>P56HFFA0HZK014503.pdf</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014404</t>
+          <t>P56HFFA0HZK014503</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -20738,7 +20738,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>D202570678 / 15052025</t>
+          <t>D202570760</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -20762,7 +20762,7 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>1834.29</v>
+        <v>2115.93</v>
       </c>
       <c r="J7" t="n">
         <v>28</v>
@@ -20784,12 +20784,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014464.pdf</t>
+          <t>P56HFFA0HZK014404.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014464</t>
+          <t>P56HFFA0HZK014404</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -20799,7 +20799,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>D202570839</t>
+          <t>D202570678 / 15052025</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -20845,12 +20845,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014503.pdf</t>
+          <t>P56HFFA0HZK014464.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014503</t>
+          <t>P56HFFA0HZK014464</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -20860,7 +20860,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>D202570760</t>
+          <t>D202570839</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -20884,7 +20884,7 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>2115.93</v>
+        <v>1834.29</v>
       </c>
       <c r="J9" t="n">
         <v>28</v>
@@ -20906,12 +20906,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014507.pdf</t>
+          <t>P56HFFA0ZZK014550.pdf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014507</t>
+          <t>P56HFFA0ZZK014550</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -20921,7 +20921,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>D202570869 / 15052025</t>
+          <t>D202570928 / 15052025</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -21028,12 +21028,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014550.pdf</t>
+          <t>P56HFFA0HZK014507.pdf</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014550</t>
+          <t>P56HFFA0HZK014507</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -21043,7 +21043,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>D202570928 / 15052025</t>
+          <t>D202570869 / 15052025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -21089,12 +21089,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014553.pdf</t>
+          <t>P56HFFA0ZZK014670.pdf</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014553</t>
+          <t>P56HFFA0ZZK014670</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -21104,7 +21104,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>D202570954 / 15052025</t>
+          <t>D202570964 / 15052025</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -21150,12 +21150,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014670.pdf</t>
+          <t>P56HFFA0ZZK014553.pdf</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014670</t>
+          <t>P56HFFA0ZZK014553</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -21165,7 +21165,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>D202570964 / 15052025</t>
+          <t>D202570954 / 15052025</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">

</xml_diff>

<commit_message>
chore: prepare for Render deployment
- Add render.yaml blueprint (free-tier web service, env vars wired)
- Add runtime.txt pinning Python 3.12.3
- Resolve unresolved README merge-conflict markers and document
  FastAPI mode + Render deploy steps
- Refresh dashboard/index.html and data/extracted.xlsx with the
  committed 315-row dataset

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/extracted.xlsx
+++ b/data/extracted.xlsx
@@ -20479,12 +20479,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>P6DED152PDA000120.pdf</t>
+          <t>P6DED152PDA000109.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>P6DED152PDA000120</t>
+          <t>P6DED152PDA000109</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -20494,7 +20494,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>D202160551</t>
+          <t>D202160528</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -20540,12 +20540,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>P6DED152PDA000109.pdf</t>
+          <t>P6DED152PDA000112.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>P6DED152PDA000109</t>
+          <t>P6DED152PDA000112</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -20555,7 +20555,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>D202160528</t>
+          <t>D202160533</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -20601,12 +20601,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>P6DED152PDA000112.pdf</t>
+          <t>P6DED152PDA000120.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>P6DED152PDA000112</t>
+          <t>P6DED152PDA000120</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -20616,7 +20616,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>D202160533</t>
+          <t>D202160551</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -20723,12 +20723,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014503.pdf</t>
+          <t>P56HFFA0HZK014404.pdf</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014503</t>
+          <t>P56HFFA0HZK014404</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -20738,7 +20738,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>D202570760</t>
+          <t>D202570678 / 15052025</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -20762,7 +20762,7 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>2115.93</v>
+        <v>1834.29</v>
       </c>
       <c r="J7" t="n">
         <v>28</v>
@@ -20784,12 +20784,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014404.pdf</t>
+          <t>P56HFFA0HZK014464.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014404</t>
+          <t>P56HFFA0HZK014464</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -20799,7 +20799,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>D202570678 / 15052025</t>
+          <t>D202570839</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -20845,12 +20845,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014464.pdf</t>
+          <t>P56HFFA0HZK014503.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014464</t>
+          <t>P56HFFA0HZK014503</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -20860,7 +20860,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>D202570839</t>
+          <t>D202570760</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -20884,7 +20884,7 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>1834.29</v>
+        <v>2115.93</v>
       </c>
       <c r="J9" t="n">
         <v>28</v>
@@ -20906,12 +20906,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014550.pdf</t>
+          <t>P56HFFA0HZK014507.pdf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014550</t>
+          <t>P56HFFA0HZK014507</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -20921,7 +20921,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>D202570928 / 15052025</t>
+          <t>D202570869 / 15052025</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -21028,12 +21028,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014507.pdf</t>
+          <t>P56HFFA0ZZK014550.pdf</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014507</t>
+          <t>P56HFFA0ZZK014550</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -21043,7 +21043,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>D202570869 / 15052025</t>
+          <t>D202570928 / 15052025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -21089,12 +21089,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014670.pdf</t>
+          <t>P56HFFA0ZZK014553.pdf</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014670</t>
+          <t>P56HFFA0ZZK014553</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -21104,7 +21104,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>D202570964 / 15052025</t>
+          <t>D202570954 / 15052025</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -21150,12 +21150,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014553.pdf</t>
+          <t>P56HFFA0ZZK014670.pdf</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014553</t>
+          <t>P56HFFA0ZZK014670</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -21165,7 +21165,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>D202570954 / 15052025</t>
+          <t>D202570964 / 15052025</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">

</xml_diff>

<commit_message>
data: upload 3005_O_432818667_00_B00.pdf [skip render]
</commit_message>
<xml_diff>
--- a/data/extracted.xlsx
+++ b/data/extracted.xlsx
@@ -20479,12 +20479,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>P6DED152PDA000109.pdf</t>
+          <t>P6DED152PDA000120.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>P6DED152PDA000109</t>
+          <t>P6DED152PDA000120</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -20494,7 +20494,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>D202160528</t>
+          <t>D202160551</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -20540,12 +20540,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>P6DED152PDA000112.pdf</t>
+          <t>P6DED152PDA000109.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>P6DED152PDA000112</t>
+          <t>P6DED152PDA000109</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -20555,7 +20555,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>D202160533</t>
+          <t>D202160528</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -20601,12 +20601,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>P6DED152PDA000120.pdf</t>
+          <t>P6DED152PDA000112.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>P6DED152PDA000120</t>
+          <t>P6DED152PDA000112</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -20616,7 +20616,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>D202160551</t>
+          <t>D202160533</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -20723,12 +20723,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014404.pdf</t>
+          <t>P56HFFA0HZK014503.pdf</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014404</t>
+          <t>P56HFFA0HZK014503</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -20738,7 +20738,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>D202570678 / 15052025</t>
+          <t>D202570760</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -20762,7 +20762,7 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>1834.29</v>
+        <v>2115.93</v>
       </c>
       <c r="J7" t="n">
         <v>28</v>
@@ -20784,12 +20784,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014464.pdf</t>
+          <t>P56HFFA0HZK014404.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014464</t>
+          <t>P56HFFA0HZK014404</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -20799,7 +20799,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>D202570839</t>
+          <t>D202570678 / 15052025</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -20845,12 +20845,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014503.pdf</t>
+          <t>P56HFFA0HZK014464.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014503</t>
+          <t>P56HFFA0HZK014464</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -20860,7 +20860,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>D202570760</t>
+          <t>D202570839</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -20884,7 +20884,7 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>2115.93</v>
+        <v>1834.29</v>
       </c>
       <c r="J9" t="n">
         <v>28</v>
@@ -20906,12 +20906,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014507.pdf</t>
+          <t>P56HFFA0ZZK014550.pdf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014507</t>
+          <t>P56HFFA0ZZK014550</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -20921,7 +20921,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>D202570869 / 15052025</t>
+          <t>D202570928 / 15052025</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -21028,12 +21028,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014550.pdf</t>
+          <t>P56HFFA0HZK014507.pdf</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014550</t>
+          <t>P56HFFA0HZK014507</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -21043,7 +21043,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>D202570928 / 15052025</t>
+          <t>D202570869 / 15052025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -21089,12 +21089,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014553.pdf</t>
+          <t>P56HFFA0ZZK014670.pdf</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014553</t>
+          <t>P56HFFA0ZZK014670</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -21104,7 +21104,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>D202570954 / 15052025</t>
+          <t>D202570964 / 15052025</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -21150,12 +21150,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014670.pdf</t>
+          <t>P56HFFA0ZZK014553.pdf</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014670</t>
+          <t>P56HFFA0ZZK014553</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -21165,7 +21165,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>D202570964 / 15052025</t>
+          <t>D202570954 / 15052025</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">

</xml_diff>

<commit_message>
data: upload MD9EMHDL24E217023.pdf [skip render]
</commit_message>
<xml_diff>
--- a/data/extracted.xlsx
+++ b/data/extracted.xlsx
@@ -17,7 +17,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Policies'!$A$1:$M$316</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Expiry Alerts (&lt;=30d)'!$A$1:$M$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Expiry Alerts (&lt;=30d)'!$A$1:$M$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'By Status'!$A$1:$C$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'By Insurer'!$A$1:$D$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'By Policy Type'!$A$1:$D$3</definedName>
@@ -989,12 +989,12 @@
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>302</t>
+          <t>301</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="H6" s="10" t="inlineStr">
@@ -20345,7 +20345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21208,8 +21208,69 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>MD9EMHDL24E217023.pdf</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>MD9EMHDL24E217023</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Royal Sundaram General Insurance Co. Limited</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>VGC1159762000101</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2025-05-28</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>accident, fire, explosion, self-ignition, lightning, theft, burglary, flood, cyclone, storm, earthquake, landslide, riot, strike, terrorism, malicious act, transit</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>7934</v>
+      </c>
+      <c r="J15" t="n">
+        <v>30</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Expiring Soon</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M14"/>
+  <autoFilter ref="A1:M15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21247,10 +21308,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C2" t="n">
-        <v>1404163</v>
+        <v>1396229</v>
       </c>
     </row>
     <row r="3">
@@ -21260,10 +21321,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C3" t="n">
-        <v>39458.31</v>
+        <v>47392.31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: upload Quectel_EC200U&EG915U_Series_AT_Commands_Manual_V1.0-1.pdf [skip render]
</commit_message>
<xml_diff>
--- a/data/extracted.xlsx
+++ b/data/extracted.xlsx
@@ -16,12 +16,12 @@
     <sheet name="By Expiry Month" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Policies'!$A$1:$M$316</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Policies'!$A$1:$M$317</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Expiry Alerts (&lt;=30d)'!$A$1:$M$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'By Status'!$A$1:$C$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'By Insurer'!$A$1:$D$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'By Policy Type'!$A$1:$D$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'By Expiry Month'!$A$1:$B$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'By Status'!$A$1:$C$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'By Insurer'!$A$1:$D$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'By Policy Type'!$A$1:$D$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'By Expiry Month'!$A$1:$B$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -329,12 +329,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'By Status'!$A$2:$A$3</f>
+              <f>'By Status'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'By Status'!$B$2:$B$3</f>
+              <f>'By Status'!$B$2:$B$4</f>
             </numRef>
           </val>
         </ser>
@@ -498,12 +498,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'By Expiry Month'!$A$2:$A$14</f>
+              <f>'By Expiry Month'!$A$2:$A$15</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'By Expiry Month'!$B$2:$B$14</f>
+              <f>'By Expiry Month'!$B$2:$B$15</f>
             </numRef>
           </val>
         </ser>
@@ -984,7 +984,7 @@
     <row r="6" ht="40" customHeight="1">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>315</t>
+          <t>316</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
@@ -1041,7 +1041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M316"/>
+  <dimension ref="A1:M317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20322,9 +20322,34 @@
         </is>
       </c>
     </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>Quectel_EC200U&amp;EG915U_Series_AT_Commands_Manual_V1.0-1.pdf</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr"/>
+      <c r="C317" t="inlineStr"/>
+      <c r="D317" t="inlineStr"/>
+      <c r="E317" t="inlineStr"/>
+      <c r="F317" t="inlineStr"/>
+      <c r="G317" t="inlineStr"/>
+      <c r="H317" t="inlineStr"/>
+      <c r="I317" t="inlineStr"/>
+      <c r="J317">
+        <f>IF(F317="","",IFERROR(INT(F317-TODAY()),""))</f>
+        <v/>
+      </c>
+      <c r="K317">
+        <f>IF(J317="","",IF(J317&lt;0,"Expired",IF(J317&lt;=30,"Expiring Soon","Active")))</f>
+        <v/>
+      </c>
+      <c r="L317" t="inlineStr"/>
+      <c r="M317" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M316"/>
-  <conditionalFormatting sqref="K2:K316">
+  <autoFilter ref="A1:M317"/>
+  <conditionalFormatting sqref="K2:K317">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Active"</formula>
     </cfRule>
@@ -20479,12 +20504,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>P6DED152PDA000109.pdf</t>
+          <t>P6DED152PDA000120.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>P6DED152PDA000109</t>
+          <t>P6DED152PDA000120</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -20494,7 +20519,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>D202160528</t>
+          <t>D202160551</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -20601,12 +20626,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>P6DED152PDA000120.pdf</t>
+          <t>P6DED152PDA000109.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>P6DED152PDA000120</t>
+          <t>P6DED152PDA000109</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -20616,7 +20641,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>D202160551</t>
+          <t>D202160528</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -20723,12 +20748,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014404.pdf</t>
+          <t>P56HFFA0HZK014507.pdf</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014404</t>
+          <t>P56HFFA0HZK014507</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -20738,7 +20763,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>D202570678 / 15052025</t>
+          <t>D202570869 / 15052025</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -20845,12 +20870,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014503.pdf</t>
+          <t>P56HFFA0HZK014404.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014503</t>
+          <t>P56HFFA0HZK014404</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -20860,7 +20885,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>D202570760</t>
+          <t>D202570678 / 15052025</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -20884,7 +20909,7 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>2115.93</v>
+        <v>1834.29</v>
       </c>
       <c r="J9" t="n">
         <v>28</v>
@@ -20906,12 +20931,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014507.pdf</t>
+          <t>P56HFFA0ZZK014670.pdf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>P56HFFA0HZK014507</t>
+          <t>P56HFFA0ZZK014670</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -20921,7 +20946,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>D202570869 / 15052025</t>
+          <t>D202570964 / 15052025</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -21028,12 +21053,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014550.pdf</t>
+          <t>P56HFFA0HZK014503.pdf</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014550</t>
+          <t>P56HFFA0HZK014503</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -21043,7 +21068,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>D202570928 / 15052025</t>
+          <t>D202570760</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -21067,7 +21092,7 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>1834.29</v>
+        <v>2115.93</v>
       </c>
       <c r="J12" t="n">
         <v>28</v>
@@ -21089,12 +21114,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014553.pdf</t>
+          <t>P56HFFA0ZZK014550.pdf</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014553</t>
+          <t>P56HFFA0ZZK014550</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -21104,7 +21129,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>D202570954 / 15052025</t>
+          <t>D202570928 / 15052025</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -21150,12 +21175,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014670.pdf</t>
+          <t>P56HFFA0ZZK014553.pdf</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>P56HFFA0ZZK014670</t>
+          <t>P56HFFA0ZZK014553</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -21165,7 +21190,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>D202570964 / 15052025</t>
+          <t>D202570954 / 15052025</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -21281,7 +21306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21327,8 +21352,21 @@
         <v>47392.31</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C3"/>
+  <autoFilter ref="A1:C4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21339,7 +21377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21492,8 +21530,18 @@
         <v>6990</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D9"/>
+  <autoFilter ref="A1:D10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21504,7 +21552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21561,8 +21609,18 @@
         <v>48915.54</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D3"/>
+  <autoFilter ref="A1:D4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21573,7 +21631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21718,8 +21776,14 @@
         <v>9</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B14"/>
+  <autoFilter ref="A1:B15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>